<commit_message>
proctoring path changes and sanitize bot changes
</commit_message>
<xml_diff>
--- a/PythonWorkingScripts_InputData/Assessment/selfassessment_report/selfassessment_generic_webreport.xlsx
+++ b/PythonWorkingScripts_InputData/Assessment/selfassessment_report/selfassessment_generic_webreport.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="10540" tabRatio="500"/>
+    <workbookView windowWidth="28800" windowHeight="10640" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1016,7 +1016,7 @@
     <t>EMPTY</t>
   </si>
   <si>
-    <t>https://s3.ap-southeast-1.amazonaws.com/test-all-hirepro-files/crpodemo/Candidates/1561290/9373ee06-e557-451a-895d-67c07fa4fef1download__1_.png</t>
+    <t>https://s3-ap-southeast-1.amazonaws.com/test-all-hirepro-files/crpodemo/Candidates/1561290/9373ee06-e557-451a-895d-67c07fa4fef1download__1_.png</t>
   </si>
   <si>
     <t>103.215.237.219</t>
@@ -1082,10 +1082,10 @@
     <t>{
   "textArea1": "I am very foodie. I love to eat. Among the number of foods, Pizza is my favourite food because it tastes and smells fabulous. My Mom cooks the best Pizzas in the world. I always ask her to make Pizza. In Pizzas, I love onion cheese Pizza a lot. This is because cheese pizza is healthy and makes me strong. To create fun we also organize pizza races in terms of who can eat the maximum number of pizzas. I can eat many pizzas at a time.",
   "capture1": [
-    "https://s3.ap-southeast-1.amazonaws.com/test-all-hirepro-files/crpodemo/testResultAnswers/20880/1561290/d61a25e6-defa-4618-886d-9633fa6c9584photoCapture0.png"
+    "https://s3-ap-southeast-1.amazonaws.com/test-all-hirepro-files/crpodemo/testResultAnswers/20880/1561290/d61a25e6-defa-4618-886d-9633fa6c9584photoCapture0.png"
   ],
   "attachment1": [
-    "https://s3.ap-southeast-1.amazonaws.com/test-all-hirepro-files/crpodemo/testResultAnswers/20880/1561290/f783bacc-d9d1-43e0-9e41-508cf06a50b6self_assessment.xls"
+    "https://s3-ap-southeast-1.amazonaws.com/test-all-hirepro-files/crpodemo/testResultAnswers/20880/1561290/f783bacc-d9d1-43e0-9e41-508cf06a50b6self_assessment.xls"
   ]
 }</t>
   </si>
@@ -1098,10 +1098,10 @@
     <t>{
   "textArea1": "I am very foodie. I love to eat. Among the number of foods, Pizza is my favourite food because it tastes and smells fabulous. My Mom cooks the best Pizzas in the world. I always ask her to make Pizza. In Pizzas, I love onion cheese Pizza a lot. This is because cheese pizza is healthy and makes me strong. To create fun we also organize pizza races in terms of who can eat the maximum number of pizzas. I can eat many pizzas at a time.",
   "capture1": [
-    "https://s3.ap-southeast-1.amazonaws.com/test-all-hirepro-files/crpodemo/testResultAnswers/20880/1561290/3efd239a-947f-43a4-a42a-ddcf47ec0e5aphotoCapture0.png"
+    "https://s3-ap-southeast-1.amazonaws.com/test-all-hirepro-files/crpodemo/testResultAnswers/20880/1561290/3efd239a-947f-43a4-a42a-ddcf47ec0e5aphotoCapture0.png"
   ],
   "attachment1": [
-    "https://s3.ap-southeast-1.amazonaws.com/test-all-hirepro-files/crpodemo/testResultAnswers/20880/1561290/6eee099d-232a-45a8-8f4e-da46f8441c46self_assessment.xls"
+    "https://s3-ap-southeast-1.amazonaws.com/test-all-hirepro-files/crpodemo/testResultAnswers/20880/1561290/6eee099d-232a-45a8-8f4e-da46f8441c46self_assessment.xls"
   ]
 }</t>
   </si>
@@ -1969,7 +1969,7 @@
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
@@ -4585,7 +4585,7 @@
     <mergeCell ref="JQ2:KG2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="H4" r:id="rId1" display="https://s3.ap-southeast-1.amazonaws.com/test-all-hirepro-files/crpodemo/Candidates/1561290/9373ee06-e557-451a-895d-67c07fa4fef1download__1_.png" tooltip="https://s3.ap-southeast-1.amazonaws.com/test-all-hirepro-files/crpodemo/Candidates/1561290/9373ee06-e557-451a-895d-67c07fa4fef1download__1_.png"/>
+    <hyperlink ref="H4" r:id="rId1" display="https://s3-ap-southeast-1.amazonaws.com/test-all-hirepro-files/crpodemo/Candidates/1561290/9373ee06-e557-451a-895d-67c07fa4fef1download__1_.png" tooltip="https://s3.ap-southeast-1.amazonaws.com/test-all-hirepro-files/crpodemo/Candidates/1561290/9373ee06-e557-451a-895d-67c07fa4fef1download__1_.png"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>